<commit_message>
PCB layout up to charging circuit
</commit_message>
<xml_diff>
--- a/Robot_BMS/BOM/Archive/Robot_BMSV1.xlsx
+++ b/Robot_BMS/BOM/Archive/Robot_BMSV1.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28723"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://computingservices-my.sharepoint.com/personal/oja37_bath_ac_uk/Documents/year 4/Group Design Business Project/PCB Design/Robot_BMS/BOM/"/>
@@ -15,7 +15,23 @@
   <sheets>
     <sheet name="Robot_BMSV1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -28,6 +44,9 @@
     <t>Value</t>
   </si>
   <si>
+    <t>Supplier</t>
+  </si>
+  <si>
     <t>Qty</t>
   </si>
   <si>
@@ -37,6 +56,12 @@
     <t>Manufacturer_Part_Number</t>
   </si>
   <si>
+    <t>Unit Price</t>
+  </si>
+  <si>
+    <t>Total Price</t>
+  </si>
+  <si>
     <t>B1,B2,B3</t>
   </si>
   <si>
@@ -64,6 +89,12 @@
     <t>GRM188R61H225KE11D</t>
   </si>
   <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Total Parts</t>
+  </si>
+  <si>
     <t>C2,C8,C9,C10,C11,C13</t>
   </si>
   <si>
@@ -142,246 +173,252 @@
     <t>4.7u</t>
   </si>
   <si>
+    <t>C19</t>
+  </si>
+  <si>
+    <t>1n</t>
+  </si>
+  <si>
+    <t>C20</t>
+  </si>
+  <si>
+    <t>180n</t>
+  </si>
+  <si>
+    <t>C21</t>
+  </si>
+  <si>
+    <t>820p</t>
+  </si>
+  <si>
+    <t>https://uk.farnell.com/kemet/c0603x821k5ractu/cap-820pf-50v-10-x7r-0603/dp/2905163</t>
+  </si>
+  <si>
+    <t>SMD Multilayer Ceramic Capacitor, 820 pF, 50 V, 0603 [1608 Metric], ± 10%, X7R</t>
+  </si>
+  <si>
+    <t>C0603X821K5RACTU</t>
+  </si>
+  <si>
+    <t>CR1,CR2,CR3</t>
+  </si>
+  <si>
+    <t>CMS05TE12L_Q_M</t>
+  </si>
+  <si>
+    <t>https://www.mouser.co.uk/ProductDetail/Toshiba/CMS05TE12LQM?qs=JiHARDETuZDcvazKO1MDNQ%3D%3D&amp;srsltid=AfmBOopWrxi0PKcgDv_hck6b5GzUq4xcRRzPONvEurGhtaMTFZsmDRz3</t>
+  </si>
+  <si>
+    <t>Schottky Diode 0.45V FWD Voltage</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>B370-13-F</t>
+  </si>
+  <si>
+    <t>https://www.diodes.com/assets/Datasheets/ds30020.pdf</t>
+  </si>
+  <si>
+    <t>Diodes Inc B370-13-F, SMT Schottky Diode, 70V 3A, 2-Pin DO-214AB</t>
+  </si>
+  <si>
+    <t>IC1</t>
+  </si>
+  <si>
+    <t>STUSB4710AQTR</t>
+  </si>
+  <si>
+    <t>https://uk.farnell.com/stmicroelectronics/stusb4710aqtr/usb-pd-controller-qfn-24/dp/2809285?srsltid=AfmBOorAHWB8haLTMyYP6OrA8XQoe2V-VsqKpObhj5T_LLLnD8WSjPc-</t>
+  </si>
+  <si>
+    <t>Super Speed PD Controller 5V/9V/12V/15V/18V/24V T/R 24-Pin QFN EP</t>
+  </si>
+  <si>
+    <t>IC2</t>
+  </si>
+  <si>
+    <t>BQ76922RSNR</t>
+  </si>
+  <si>
+    <t>https://www.mouser.co.uk/ProductDetail/Texas-Instruments/BQ76922RSNR?qs=dbcCsuKDzFV1TGwm4B7DLw%3D%3D&amp;srsltid=AfmBOor1BwixVM4imBs0xd3ssBI2snkv_dKEs7gEDBC8HCYSlzWdYF-s</t>
+  </si>
+  <si>
+    <t>Battery Management Three-series to five-series cell lithium-ion and lithium-phosphate battery monitor</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>https://uk.farnell.com/wurth-elektronik/632723300011/usb-connector-3-1-type-c-rcpt/dp/2984361?srsltid=AfmBOoq_rsfBg-e4OV9-XtGNTpMTNYyO152eWN8LegmEdX5MT1hYTNFv</t>
+  </si>
+  <si>
+    <t>USB Connectors WR-COM USB3.1 Type C SuperSpeed+ Rcpt</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>Conn_01x14_Pin</t>
+  </si>
+  <si>
+    <t>https://www.digikey.co.uk/en/products/detail/w-rth-elektronik/61301411121/4846849?gclsrc=aw.ds&amp;&amp;utm_adgroup=&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=PMax%20Shopping_Product_New%20Customer%20Acquisition&amp;utm_term=&amp;productid=4846849&amp;utm_content=&amp;utm_id=go_cmp-19905262708_adg-_ad-__dev-c_ext-_prd-4846849_sig-Cj0KCQjw1um-BhDtARIsABjU5x5IZchPm1Re5jb8lZ6dm-_WGVxZLQDpy4bDA0Enw1KwuXt_1ODZSgUaAiIqEALw_wcB&amp;gad_source=1&amp;gclid=Cj0KCQjw1um-BhDtARIsABjU5x5IZchPm1Re5jb8lZ6dm-_WGVxZLQDpy4bDA0Enw1KwuXt_1ODZSgUaAiIqEALw_wcB&amp;gclsrc=aw.ds</t>
+  </si>
+  <si>
+    <t>Generic connector, single row, 01x14, script generated</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/6941xx301002.pdf</t>
+  </si>
+  <si>
+    <t>DC Power Jack Right Angled 5A, 30 V(DC), Contact Resistance 50 m</t>
+  </si>
+  <si>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>ETQ-P5M220YSC</t>
+  </si>
+  <si>
+    <t>https://industrial.panasonic.com/cdbs/www-data/pdf/AGL0000/AGL0000C70.pdf</t>
+  </si>
+  <si>
+    <t>Series/Type: High Vibration Acceleration-resistant Power Choke Coil for Automotive-MS (MC type), Size [L] (mm): 10.910.0, Height (mm): 5.6, Inductance (H): 20, DC Resistance [Typ.] (at 20) (m): 45.5, DC Resistance [max.] (at 20) (m): 50, Rated Current [Typ.] (T=40K, FR4, t=1.6 mm,Four-layer PWB) (A): 5.2, Rated Current [Typ.] (T=40K, High heat dissipation PWB) (A): 6.2, Rated Current [Typ.] (L=30%)  (A): 7.9, Weight (Typ.) (g): 3.1, AEC-Q200 compliant</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>MSD1583-223MEB</t>
+  </si>
+  <si>
+    <t>INDUCTOR, 22UH, 3.45A, 20%, PWR, 10.5MHZ</t>
+  </si>
+  <si>
+    <t>Q1,Q3</t>
+  </si>
+  <si>
+    <t>2N7002</t>
+  </si>
+  <si>
+    <t>https://www.mouser.co.uk/ProductDetail/Infineon-Technologies/2N7002-H6327?qs=CVg1V728NXGZyf6kD1tkzQ%3D%3D&amp;mgh=1&amp;vip=1&amp;utm_id=20808080842&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_marketing_tactic=emeacorp&amp;gad_source=1&amp;gclid=Cj0KCQjw1um-BhDtARIsABjU5x70kCIU17Y9chiVxNH_Vom0j4sKZ5ToqWr6DV3ByRFWQx4h5b8ahzcaAj4GEALw_wcB</t>
+  </si>
+  <si>
+    <t>0.115A Id, 60V Vds, N-Channel MOSFET, SOT-23</t>
+  </si>
+  <si>
+    <t>2N7002 H6327</t>
+  </si>
+  <si>
+    <t>Q2,Q4</t>
+  </si>
+  <si>
+    <t>SIS413DN-T1-GE3</t>
+  </si>
+  <si>
+    <t>https://www.mouser.co.uk/ProductDetail/Vishay-Semiconductors/SIS413DN-T1-GE3?qs=vgn07B5hXav8x6TX%252BtAIoQ%3D%3D</t>
+  </si>
+  <si>
+    <t>P-Ch PowerPAK1212 Cu 30V 9.4mohm@10V</t>
+  </si>
+  <si>
+    <t>R1,R2,R3</t>
+  </si>
+  <si>
+    <t>3k24</t>
+  </si>
+  <si>
+    <t>https://www.digikey.co.uk/en/products/detail/yageo/RC0603FR-073K24L/727125</t>
+  </si>
+  <si>
+    <t>RES 3.24K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>RC0603FR-073K24L</t>
+  </si>
+  <si>
+    <t>R4,R26</t>
+  </si>
+  <si>
+    <t>100k</t>
+  </si>
+  <si>
+    <t>https://www.digikey.co.uk/en/products/detail/rohm-semiconductor/ESR03EZPF1003/1983430</t>
+  </si>
+  <si>
+    <t>RES 100K OHM 1% 1/4W 0603</t>
+  </si>
+  <si>
+    <t>ESR03EZPF1003</t>
+  </si>
+  <si>
+    <t>R5</t>
+  </si>
+  <si>
+    <t>4.81k</t>
+  </si>
+  <si>
+    <t>https://www.mouser.co.uk/ProductDetail/KOA-Speer/RN73H1JTTD4811B25?qs=582LK1XNA7LTNwR5VHugwg%3D%3D&amp;srsltid=AfmBOoo6gri6g2xu2rXc1ABkOav6S-9c3aTxtg7NNutX6ztjQHESnNk1</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 4.81kOhm,0603,0.1%,2</t>
+  </si>
+  <si>
+    <t>RN73H1JTTD4811B25</t>
+  </si>
+  <si>
+    <t>R6,R8,R18,R22,R27</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>1k</t>
+  </si>
+  <si>
+    <t>https://www.digikey.co.uk/en/products/detail/vishay-dale/CRCW06031K00JNEAIF/3477274?srsltid=AfmBOoqM_C78zLfiw-YdUpmN3JS4P2_NqO2IPeLygIKGkpOp0cehDR8Q</t>
+  </si>
+  <si>
+    <t>RES SMD 1K OHM 5% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>CRCW06031K00JNEAIF</t>
+  </si>
+  <si>
+    <t>R9,R10,R11,R12,R16,R19</t>
+  </si>
+  <si>
+    <t>R14,R17</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>https://www.digikey.co.uk/en/products/detail/yageo/RC0603FR-0710KL/726880?srsltid=AfmBOoqjqC5qo52Z-BfREj56jdcNCkiFl9EdC8LTCxkmf6IG3DRH4_a1</t>
+  </si>
+  <si>
+    <t>10 kOhms Â±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>R15</t>
+  </si>
+  <si>
+    <t>1 mOhm</t>
+  </si>
+  <si>
+    <t>R20</t>
+  </si>
+  <si>
     <t>None</t>
   </si>
   <si>
-    <t>C19</t>
-  </si>
-  <si>
-    <t>1n</t>
-  </si>
-  <si>
-    <t>C20</t>
-  </si>
-  <si>
-    <t>180n</t>
-  </si>
-  <si>
-    <t>C21</t>
-  </si>
-  <si>
-    <t>820p</t>
-  </si>
-  <si>
-    <t>C0603X821K5RACTU</t>
-  </si>
-  <si>
-    <t>CR1,CR2,CR3</t>
-  </si>
-  <si>
-    <t>CMS05TE12L_Q_M</t>
-  </si>
-  <si>
-    <t>https://www.mouser.co.uk/ProductDetail/Toshiba/CMS05TE12LQM?qs=JiHARDETuZDcvazKO1MDNQ%3D%3D&amp;srsltid=AfmBOopWrxi0PKcgDv_hck6b5GzUq4xcRRzPONvEurGhtaMTFZsmDRz3</t>
-  </si>
-  <si>
-    <t>Schottky Diode 0.45V FWD Voltage</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>B370-13-F</t>
-  </si>
-  <si>
-    <t>https://www.diodes.com/assets/Datasheets/ds30020.pdf</t>
-  </si>
-  <si>
-    <t>Diodes Inc B370-13-F, SMT Schottky Diode, 70V 3A, 2-Pin DO-214AB</t>
-  </si>
-  <si>
-    <t>IC1</t>
-  </si>
-  <si>
-    <t>STUSB4710AQTR</t>
-  </si>
-  <si>
-    <t>https://uk.farnell.com/stmicroelectronics/stusb4710aqtr/usb-pd-controller-qfn-24/dp/2809285?srsltid=AfmBOorAHWB8haLTMyYP6OrA8XQoe2V-VsqKpObhj5T_LLLnD8WSjPc-</t>
-  </si>
-  <si>
-    <t>Super Speed PD Controller 5V/9V/12V/15V/18V/24V T/R 24-Pin QFN EP</t>
-  </si>
-  <si>
-    <t>IC2</t>
-  </si>
-  <si>
-    <t>BQ76922RSNR</t>
-  </si>
-  <si>
-    <t>https://www.mouser.co.uk/ProductDetail/Texas-Instruments/BQ76922RSNR?qs=dbcCsuKDzFV1TGwm4B7DLw%3D%3D&amp;srsltid=AfmBOor1BwixVM4imBs0xd3ssBI2snkv_dKEs7gEDBC8HCYSlzWdYF-s</t>
-  </si>
-  <si>
-    <t>Battery Management Three-series to five-series cell lithium-ion and lithium-phosphate battery monitor</t>
-  </si>
-  <si>
-    <t>J1</t>
-  </si>
-  <si>
-    <t>https://uk.farnell.com/wurth-elektronik/632723300011/usb-connector-3-1-type-c-rcpt/dp/2984361?srsltid=AfmBOoq_rsfBg-e4OV9-XtGNTpMTNYyO152eWN8LegmEdX5MT1hYTNFv</t>
-  </si>
-  <si>
-    <t>USB Connectors WR-COM USB3.1 Type C SuperSpeed+ Rcpt</t>
-  </si>
-  <si>
-    <t>J2</t>
-  </si>
-  <si>
-    <t>Conn_01x14_Pin</t>
-  </si>
-  <si>
-    <t>https://www.digikey.co.uk/en/products/detail/w-rth-elektronik/61301411121/4846849?gclsrc=aw.ds&amp;&amp;utm_adgroup=&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=PMax%20Shopping_Product_New%20Customer%20Acquisition&amp;utm_term=&amp;productid=4846849&amp;utm_content=&amp;utm_id=go_cmp-19905262708_adg-_ad-__dev-c_ext-_prd-4846849_sig-Cj0KCQjw1um-BhDtARIsABjU5x5IZchPm1Re5jb8lZ6dm-_WGVxZLQDpy4bDA0Enw1KwuXt_1ODZSgUaAiIqEALw_wcB&amp;gad_source=1&amp;gclid=Cj0KCQjw1um-BhDtARIsABjU5x5IZchPm1Re5jb8lZ6dm-_WGVxZLQDpy4bDA0Enw1KwuXt_1ODZSgUaAiIqEALw_wcB&amp;gclsrc=aw.ds</t>
-  </si>
-  <si>
-    <t>Generic connector, single row, 01x14, script generated</t>
-  </si>
-  <si>
-    <t>J3</t>
-  </si>
-  <si>
-    <t>https://www.we-online.com/components/products/datasheet/6941xx301002.pdf</t>
-  </si>
-  <si>
-    <t>DC Power Jack Right Angled 5A, 30 V(DC), Contact Resistance 50 m</t>
-  </si>
-  <si>
-    <t>J4</t>
-  </si>
-  <si>
-    <t>L1</t>
-  </si>
-  <si>
-    <t>ETQ-P5M220YSC</t>
-  </si>
-  <si>
-    <t>https://industrial.panasonic.com/cdbs/www-data/pdf/AGL0000/AGL0000C70.pdf</t>
-  </si>
-  <si>
-    <t>Series/Type: High Vibration Acceleration-resistant Power Choke Coil for Automotive-MS (MC type), Size [L] (mm): 10.910.0, Height (mm): 5.6, Inductance (H): 20, DC Resistance [Typ.] (at 20) (m): 45.5, DC Resistance [max.] (at 20) (m): 50, Rated Current [Typ.] (T=40K, FR4, t=1.6 mm,Four-layer PWB) (A): 5.2, Rated Current [Typ.] (T=40K, High heat dissipation PWB) (A): 6.2, Rated Current [Typ.] (L=30%)  (A): 7.9, Weight (Typ.) (g): 3.1, AEC-Q200 compliant</t>
-  </si>
-  <si>
-    <t>L2</t>
-  </si>
-  <si>
-    <t>MSD1583-223MEB</t>
-  </si>
-  <si>
-    <t>INDUCTOR, 22UH, 3.45A, 20%, PWR, 10.5MHZ</t>
-  </si>
-  <si>
-    <t>Q1,Q3</t>
-  </si>
-  <si>
-    <t>2N7002</t>
-  </si>
-  <si>
-    <t>https://www.mouser.co.uk/ProductDetail/Infineon-Technologies/2N7002-H6327?qs=CVg1V728NXGZyf6kD1tkzQ%3D%3D&amp;mgh=1&amp;vip=1&amp;utm_id=20808080842&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_marketing_tactic=emeacorp&amp;gad_source=1&amp;gclid=Cj0KCQjw1um-BhDtARIsABjU5x70kCIU17Y9chiVxNH_Vom0j4sKZ5ToqWr6DV3ByRFWQx4h5b8ahzcaAj4GEALw_wcB</t>
-  </si>
-  <si>
-    <t>0.115A Id, 60V Vds, N-Channel MOSFET, SOT-23</t>
-  </si>
-  <si>
-    <t>2N7002 H6327</t>
-  </si>
-  <si>
-    <t>Q2,Q4</t>
-  </si>
-  <si>
-    <t>SIS413DN-T1-GE3</t>
-  </si>
-  <si>
-    <t>https://www.mouser.co.uk/ProductDetail/Vishay-Semiconductors/SIS413DN-T1-GE3?qs=vgn07B5hXav8x6TX%252BtAIoQ%3D%3D</t>
-  </si>
-  <si>
-    <t>P-Ch PowerPAK1212 Cu 30V 9.4mohm@10V</t>
-  </si>
-  <si>
-    <t>R1,R2,R3</t>
-  </si>
-  <si>
-    <t>3k24</t>
-  </si>
-  <si>
-    <t>https://www.digikey.co.uk/en/products/detail/yageo/RC0603FR-073K24L/727125</t>
-  </si>
-  <si>
-    <t>RES 3.24K OHM 1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>RC0603FR-073K24L</t>
-  </si>
-  <si>
-    <t>R4,R26</t>
-  </si>
-  <si>
-    <t>100k</t>
-  </si>
-  <si>
-    <t>https://www.digikey.co.uk/en/products/detail/rohm-semiconductor/ESR03EZPF1003/1983430</t>
-  </si>
-  <si>
-    <t>RES 100K OHM 1% 1/4W 0603</t>
-  </si>
-  <si>
-    <t>ESR03EZPF1003</t>
-  </si>
-  <si>
-    <t>R5</t>
-  </si>
-  <si>
-    <t>4.81k</t>
-  </si>
-  <si>
-    <t>https://www.mouser.co.uk/ProductDetail/KOA-Speer/RN73H1JTTD4811B25?qs=582LK1XNA7LTNwR5VHugwg%3D%3D&amp;srsltid=AfmBOoo6gri6g2xu2rXc1ABkOav6S-9c3aTxtg7NNutX6ztjQHESnNk1</t>
-  </si>
-  <si>
-    <t>Thin Film Resistors - SMD 4.81kOhm,0603,0.1%,2</t>
-  </si>
-  <si>
-    <t>RN73H1JTTD4811B25</t>
-  </si>
-  <si>
-    <t>R6,R8,R18,R22,R27</t>
-  </si>
-  <si>
-    <t>R7</t>
-  </si>
-  <si>
-    <t>1k</t>
-  </si>
-  <si>
-    <t>https://www.digikey.co.uk/en/products/detail/vishay-dale/CRCW06031K00JNEAIF/3477274?srsltid=AfmBOoqM_C78zLfiw-YdUpmN3JS4P2_NqO2IPeLygIKGkpOp0cehDR8Q</t>
-  </si>
-  <si>
-    <t>RES SMD 1K OHM 5% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>CRCW06031K00JNEAIF</t>
-  </si>
-  <si>
-    <t>R9,R10,R11,R12,R16,R19</t>
-  </si>
-  <si>
-    <t>R14,R17</t>
-  </si>
-  <si>
-    <t>10k</t>
-  </si>
-  <si>
-    <t>https://www.digikey.co.uk/en/products/detail/yageo/RC0603FR-0710KL/726880?srsltid=AfmBOoqjqC5qo52Z-BfREj56jdcNCkiFl9EdC8LTCxkmf6IG3DRH4_a1</t>
-  </si>
-  <si>
-    <t>10 kOhms Â±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
-  </si>
-  <si>
-    <t>R15</t>
-  </si>
-  <si>
-    <t>1 mOhm</t>
-  </si>
-  <si>
-    <t>R20</t>
-  </si>
-  <si>
     <t>R21</t>
   </si>
   <si>
@@ -473,27 +510,6 @@
   </si>
   <si>
     <t>CSD18563Q5A</t>
-  </si>
-  <si>
-    <t>Supplier</t>
-  </si>
-  <si>
-    <t>Total Parts</t>
-  </si>
-  <si>
-    <t>Cost</t>
-  </si>
-  <si>
-    <t>SMD Multilayer Ceramic Capacitor, 820 pF, 50 V, 0603 [1608 Metric], ± 10%, X7R</t>
-  </si>
-  <si>
-    <t>https://uk.farnell.com/kemet/c0603x821k5ractu/cap-820pf-50v-10-x7r-0603/dp/2905163</t>
-  </si>
-  <si>
-    <t>Total Price</t>
-  </si>
-  <si>
-    <t>Unit Price</t>
   </si>
 </sst>
 </file>
@@ -501,9 +517,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1008,22 +1024,20 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1403,7 +1417,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90A36E9A-12F6-4CAD-99D7-388F0B49B123}">
   <dimension ref="A1:K44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
     <col min="2" max="2" width="22.28515625" customWidth="1"/>
@@ -1415,7 +1429,7 @@
     <col min="11" max="11" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1423,231 +1437,231 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>151</v>
+        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>157</v>
+        <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="60">
       <c r="A2" s="4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D2" s="4">
         <v>3</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G2" s="4">
         <v>3.08</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H2" s="4">
         <f>G2*D2</f>
         <v>9.24</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="60">
       <c r="A3" s="4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D3" s="4">
         <v>3</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G3" s="4">
         <v>0.22</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="4">
         <f t="shared" ref="H3:H44" si="0">G3*D3</f>
         <v>0.66</v>
       </c>
-      <c r="J3" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="J3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="45">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D4" s="4">
         <v>6</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G4" s="4">
         <v>0.05</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="4">
         <f t="shared" si="0"/>
         <v>0.30000000000000004</v>
       </c>
-      <c r="J4" s="8" t="e">
+      <c r="J4" s="6" t="e">
         <f>SUM(H2:H44)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="4">
         <f>SUM(D2:D44)</f>
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="30">
       <c r="A5" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D5" s="4">
         <v>4</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="G5" s="4">
         <v>0.11</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="4">
         <f t="shared" si="0"/>
         <v>0.44</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11">
       <c r="A6" s="4" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D6" s="4">
         <v>4</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="G6" s="4">
         <v>0.156</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="4">
         <f t="shared" si="0"/>
         <v>0.624</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11">
       <c r="A7" s="4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="4">
         <v>2</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G7" s="4">
         <v>0.20399999999999999</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="4">
         <f t="shared" si="0"/>
         <v>0.40799999999999997</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="45">
       <c r="A8" s="4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D8" s="4">
         <v>1</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="G8" s="4">
         <v>0.156</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="4">
         <f t="shared" si="0"/>
         <v>0.156</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11">
       <c r="A9" s="4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="4">
@@ -1656,17 +1670,17 @@
       <c r="E9" s="5"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="6">
+      <c r="H9" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11">
       <c r="A10" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="4">
@@ -1675,17 +1689,17 @@
       <c r="E10" s="5"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
-      <c r="H10" s="6">
+      <c r="H10" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11">
       <c r="A11" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="4">
@@ -1694,159 +1708,159 @@
       <c r="E11" s="5"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
-      <c r="H11" s="6">
+      <c r="H11" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="30">
       <c r="A12" s="4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>155</v>
+        <v>51</v>
       </c>
       <c r="D12" s="4">
         <v>1</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>53</v>
       </c>
       <c r="G12" s="4">
         <v>9.5000000000000001E-2</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="4">
         <f t="shared" si="0"/>
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="45">
       <c r="A13" s="4" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D13" s="4">
         <v>3</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="G13" s="4">
         <v>0.8</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="4">
         <f t="shared" si="0"/>
         <v>2.4000000000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="30">
       <c r="A14" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D14" s="4">
         <v>1</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G14" s="4"/>
-      <c r="H14" s="6">
+      <c r="H14" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="45">
       <c r="A15" s="4" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D15" s="4">
         <v>1</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="G15" s="4">
         <v>1.03</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="4">
         <f t="shared" si="0"/>
         <v>1.03</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="45">
       <c r="A16" s="4" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D16" s="4">
         <v>1</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G16" s="4">
         <v>3.08</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="4">
         <f t="shared" si="0"/>
         <v>3.08</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="45">
       <c r="A17" s="4" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B17" s="4">
         <v>632723300011</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D17" s="4">
         <v>1</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F17" s="4">
         <v>632723300011</v>
@@ -1854,26 +1868,26 @@
       <c r="G17" s="4">
         <v>3.62</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="4">
         <f t="shared" si="0"/>
         <v>3.62</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="135">
       <c r="A18" s="4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D18" s="4">
         <v>1</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F18" s="4">
         <v>61301411121</v>
@@ -1881,39 +1895,39 @@
       <c r="G18" s="4">
         <v>0.67</v>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="4">
         <f t="shared" si="0"/>
         <v>0.67</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="30">
       <c r="A19" s="4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B19" s="4">
         <v>694108301002</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="D19" s="4">
         <v>1</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="F19" s="4">
         <v>694108301002</v>
       </c>
       <c r="G19" s="4"/>
-      <c r="H19" s="6">
+      <c r="H19" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="4" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B20" s="4">
         <v>691137710002</v>
@@ -1925,253 +1939,253 @@
       <c r="E20" s="5"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
-      <c r="H20" s="6">
+      <c r="H20" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="195" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="195">
       <c r="A21" s="4" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D21" s="4">
         <v>1</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="G21" s="4">
         <v>1.2</v>
       </c>
-      <c r="H21" s="6">
+      <c r="H21" s="4">
         <f t="shared" si="0"/>
         <v>1.2</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="30">
       <c r="A22" s="4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="4">
         <v>1</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G22" s="4"/>
-      <c r="H22" s="6">
+      <c r="H22" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="90">
       <c r="A23" s="4" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D23" s="4">
         <v>2</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="G23" s="4">
         <v>0.21</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="4">
         <f t="shared" si="0"/>
         <v>0.42</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="30">
       <c r="A24" s="4" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D24" s="4">
         <v>2</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="G24" s="4">
         <v>0.57999999999999996</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="4">
         <f t="shared" si="0"/>
         <v>1.1599999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="30">
       <c r="A25" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D25" s="4">
         <v>3</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G25" s="4">
         <v>0.08</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="4">
         <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="30">
       <c r="A26" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D26" s="4">
         <v>2</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G26" s="4">
         <v>0.12</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="4">
         <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="45">
       <c r="A27" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D27" s="4">
         <v>1</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="G27" s="4">
         <v>0.18</v>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="4">
         <f t="shared" si="0"/>
         <v>0.18</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8">
       <c r="A28" s="4" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B28" s="4">
         <v>100</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D28" s="4">
         <v>5</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H28" s="6" t="e">
+        <v>31</v>
+      </c>
+      <c r="H28" s="4" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="45">
       <c r="A29" s="4" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="D29" s="4">
         <v>1</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="G29" s="4">
         <v>0.33600000000000002</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="4">
         <f t="shared" si="0"/>
         <v>0.33600000000000002</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8">
       <c r="A30" s="4" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B30" s="4">
         <v>20</v>
@@ -2181,53 +2195,53 @@
         <v>6</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H30" s="6" t="e">
+        <v>31</v>
+      </c>
+      <c r="H30" s="4" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="45">
       <c r="A31" s="4" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="D31" s="4">
         <v>2</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4">
         <v>9.6000000000000002E-2</v>
       </c>
-      <c r="H31" s="6">
+      <c r="H31" s="4">
         <f t="shared" si="0"/>
         <v>0.192</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8">
       <c r="A32" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D32" s="4">
         <v>1</v>
@@ -2235,14 +2249,14 @@
       <c r="E32" s="5"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
-      <c r="H32" s="6">
+      <c r="H32" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8">
       <c r="A33" s="4" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B33" s="4">
         <v>604</v>
@@ -2254,19 +2268,19 @@
       <c r="E33" s="5"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H33" s="6" t="e">
+        <v>126</v>
+      </c>
+      <c r="H33" s="4" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8">
       <c r="A34" s="4" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="4">
@@ -2275,42 +2289,42 @@
       <c r="E34" s="5"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H34" s="6" t="e">
+        <v>126</v>
+      </c>
+      <c r="H34" s="4" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="30">
       <c r="A35" s="4" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="D35" s="4">
         <v>1</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
-      <c r="H35" s="6">
+      <c r="H35" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8">
       <c r="A36" s="4" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="4">
@@ -2319,165 +2333,165 @@
       <c r="E36" s="5"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H36" s="6" t="e">
+        <v>126</v>
+      </c>
+      <c r="H36" s="4" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="90">
       <c r="A37" s="4" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="D37" s="4">
         <v>3</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="G37" s="4">
         <v>0.45</v>
       </c>
-      <c r="H37" s="6">
+      <c r="H37" s="4">
         <f t="shared" si="0"/>
         <v>1.35</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8">
       <c r="A38" s="4" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D38" s="4">
         <v>2</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
-      <c r="H38" s="6">
+      <c r="H38" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8">
       <c r="A39" s="4" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D39" s="4">
         <v>2</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
-      <c r="H39" s="6">
+      <c r="H39" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8">
       <c r="A40" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D40" s="4">
         <v>2</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
-      <c r="H40" s="6">
+      <c r="H40" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8">
       <c r="A41" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B41" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>142</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>135</v>
       </c>
       <c r="D41" s="4">
         <v>1</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
-      <c r="H41" s="6">
+      <c r="H41" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="60">
       <c r="A42" s="4" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="D42" s="4">
         <v>1</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="G42" s="4">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H42" s="6">
+      <c r="H42" s="4">
         <f t="shared" si="0"/>
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8">
       <c r="A43" s="4" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="4">
@@ -2486,20 +2500,20 @@
       <c r="E43" s="5"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
-      <c r="H43" s="6">
+      <c r="H43" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8">
       <c r="A44" s="4" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="D44" s="4">
         <v>1</v>
@@ -2507,7 +2521,7 @@
       <c r="E44" s="5"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
-      <c r="H44" s="6">
+      <c r="H44" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>

</xml_diff>